<commit_message>
W03 D5 workbooks after pass 4: the roster flags an empty slot and a draw position outside 1 to 9, keeps card 10 from the billing groups, reads the new minutes and ships Monday's Option B as its example; the scoring sheet names a cleared Sat cell instead of counting -1 learners
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E7dQAECPqF2d5xd5HAQYwz
</commit_message>
<xml_diff>
--- a/content/W03/D5/gd/C2_W03_D05_gd_roster_TRAINER.xlsx
+++ b/content/W03/D5/gd/C2_W03_D05_gd_roster_TRAINER.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="119">
   <si>
     <t xml:space="preserve">Build 1 GD roster, Friday and Saturday morning (TRAINER ONLY)</t>
   </si>
@@ -45,10 +45,13 @@
     <t xml:space="preserve">At the Friday opening, the Programme Head draws the GD order by lot and types each group's position on Inputs. Slot 1 is the first round; the card each slot carries is fixed on Roster, so complexity climbs with the slot.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cards 07 to 10 read for four minutes and discuss for seventeen; cards 01 to 06 read for three and discuss for eighteen. Every round is 30 minutes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check reads the result: the GD minutes, how the roster stretches for more groups, whether every round ends inside its block, and whether any group meets a card it is kept from.</t>
+    <t xml:space="preserve">Cards 01 to 04 read for four minutes and discuss for seventeen, cards 05 to 08 read for five and discuss for sixteen, and cards 09 and 10 read for six and discuss for fifteen. Every round is 30 minutes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check reads the result: the GD minutes, how the roster stretches for more groups, whether every round ends inside its block, whether any group meets a card it is kept from, whether every slot has a group drawn, and whether every draw position is between 1 and 9.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The roster seats nine groups. With more, change the group count on Inputs to read the stretch on Check, and seat each extra round by hand in the time Check names.</t>
   </si>
   <si>
     <t xml:space="preserve">A clash means swapping the card with the other card of the same level on Roster, if that card's own flag allows, or with the spare, card 08, which is kept from nobody.</t>
@@ -165,10 +168,10 @@
     <t xml:space="preserve">none</t>
   </si>
   <si>
-    <t xml:space="preserve">3, then 18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Should Kalpa stop posting paper statements and bill patients by text and email only?</t>
+    <t xml:space="preserve">4, then 17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should Kalpa stop mailing paper statements and bill patients by text and email only?</t>
   </si>
   <si>
     <t xml:space="preserve">Should Kalpa promise same-day results in all six metros?</t>
@@ -183,6 +186,9 @@
     <t xml:space="preserve">3 and 5</t>
   </si>
   <si>
+    <t xml:space="preserve">5, then 16</t>
+  </si>
+  <si>
     <t xml:space="preserve">Should the lab director rank the six labs monthly on turnaround?</t>
   </si>
   <si>
@@ -192,9 +198,6 @@
     <t xml:space="preserve">Where should the board's $2 million for growth go?</t>
   </si>
   <si>
-    <t xml:space="preserve">4, then 17</t>
-  </si>
-  <si>
     <t xml:space="preserve">Should Kalpa sign the plan's preferred-lab offer in Dallas? (the spare)</t>
   </si>
   <si>
@@ -204,6 +207,9 @@
     <t xml:space="preserve">3</t>
   </si>
   <si>
+    <t xml:space="preserve">6, then 15</t>
+  </si>
+  <si>
     <t xml:space="preserve">Should Kalpa move its Texas Medicaid claim work to Bengaluru?</t>
   </si>
   <si>
@@ -364,6 +370,18 @@
   </si>
   <si>
     <t xml:space="preserve">Groups drawn to one slot each</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slots with no group drawn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot verdict</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draw positions outside 1 to 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Position verdict</t>
   </si>
 </sst>
 </file>
@@ -744,7 +762,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -780,12 +798,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -793,6 +811,11 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -821,105 +844,105 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>30</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>180</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>3</v>
@@ -930,7 +953,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>3</v>
@@ -941,7 +964,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>1</v>
@@ -952,7 +975,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>1</v>
@@ -963,7 +986,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>2</v>
@@ -974,10 +997,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>6</v>
@@ -985,10 +1008,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>7</v>
@@ -996,10 +1019,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>8</v>
@@ -1007,10 +1030,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B21" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>9</v>
@@ -1050,24 +1073,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1075,16 +1098,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1092,16 +1115,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1109,16 +1132,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1126,16 +1149,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1143,16 +1166,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1160,16 +1183,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1177,16 +1200,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1194,16 +1217,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1211,16 +1234,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1228,16 +1251,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1276,54 +1299,54 @@
   <sheetData>
     <row r="1" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1331,19 +1354,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G4" s="2" t="n">
         <f aca="false">Inputs!$B$4</f>
@@ -1386,19 +1409,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G5" s="2" t="n">
         <f aca="false">Inputs!$B$4</f>
@@ -1441,19 +1464,19 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G6" s="2" t="n">
         <f aca="false">Inputs!$B$4+Inputs!$B$3</f>
@@ -1496,19 +1519,19 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G7" s="2" t="n">
         <f aca="false">Inputs!$B$4+Inputs!$B$3</f>
@@ -1551,19 +1574,19 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G8" s="2" t="n">
         <f aca="false">Inputs!$B$4+2*Inputs!$B$3</f>
@@ -1606,19 +1629,19 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G9" s="2" t="n">
         <f aca="false">Inputs!$B$4+3*Inputs!$B$3</f>
@@ -1641,7 +1664,7 @@
       </c>
       <c r="L9" s="2" t="n">
         <f aca="false">IFERROR(INDEX(Inputs!$B$13:$B$21,MATCH(K9,Inputs!$A$13:$A$21,0)),"")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M9" s="2" t="str">
         <f aca="false">INDEX(Prompts!$D$3:$D$12,MATCH(J9,Prompts!$A$3:$A$12,0))</f>
@@ -1661,19 +1684,19 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G10" s="2" t="n">
         <f aca="false">Inputs!$B$4+4*Inputs!$B$3</f>
@@ -1696,7 +1719,7 @@
       </c>
       <c r="L10" s="2" t="n">
         <f aca="false">IFERROR(INDEX(Inputs!$B$13:$B$21,MATCH(K10,Inputs!$A$13:$A$21,0)),"")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" s="2" t="str">
         <f aca="false">INDEX(Prompts!$D$3:$D$12,MATCH(J10,Prompts!$A$3:$A$12,0))</f>
@@ -1716,19 +1739,19 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G11" s="2" t="n">
         <f aca="false">0</f>
@@ -1751,7 +1774,7 @@
       </c>
       <c r="L11" s="2" t="n">
         <f aca="false">IFERROR(INDEX(Inputs!$B$13:$B$21,MATCH(K11,Inputs!$A$13:$A$21,0)),"")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M11" s="2" t="str">
         <f aca="false">INDEX(Prompts!$D$3:$D$12,MATCH(J11,Prompts!$A$3:$A$12,0))</f>
@@ -1771,19 +1794,19 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="G12" s="2" t="n">
         <f aca="false">0</f>
@@ -1806,11 +1829,11 @@
       </c>
       <c r="L12" s="2" t="n">
         <f aca="false">IFERROR(INDEX(Inputs!$B$13:$B$21,MATCH(K12,Inputs!$A$13:$A$21,0)),"")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M12" s="2" t="str">
         <f aca="false">INDEX(Prompts!$D$3:$D$12,MATCH(J12,Prompts!$A$3:$A$12,0))</f>
-        <v>none</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="str">
         <f aca="false">IF(L12="","no group",IF(ISNUMBER(SEARCH(L12,M12)),"swap: the card meets the group's own sub-problem","ok"))</f>
@@ -1823,12 +1846,12 @@
     </row>
     <row r="15" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1857,12 +1880,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>3</v>
@@ -1870,7 +1893,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>30</v>
@@ -1878,7 +1901,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>20</v>
@@ -1886,7 +1909,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>3</v>
@@ -1894,7 +1917,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>10</v>
@@ -1902,21 +1925,21 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B10" s="2" t="n">
         <f aca="false">B3*B4</f>
@@ -1933,7 +1956,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B11" s="2" t="n">
         <f aca="false">B5</f>
@@ -1950,7 +1973,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B12" s="2" t="n">
         <f aca="false">B6*Inputs!B6</f>
@@ -1967,7 +1990,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B13" s="2" t="n">
         <f aca="false">B7</f>
@@ -1984,7 +2007,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B14" s="2" t="n">
         <f aca="false">Inputs!B5-SUM(B10:B13)</f>
@@ -2001,7 +2024,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B16" s="2" t="str">
         <f aca="false">IF(B14&lt;0,"block two runs over by "&amp;-B14&amp;" minutes: shorten the tranche","block two fits with "&amp;B14&amp;" minutes of slack")</f>
@@ -2024,7 +2047,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -2033,20 +2056,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B3" s="2" t="n">
         <f aca="false">Inputs!B6*Inputs!B3</f>
@@ -2055,7 +2078,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B4" s="2" t="n">
         <f aca="false">INT((Inputs!B5-Inputs!B4)/Inputs!B3)</f>
@@ -2064,7 +2087,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B5" s="2" t="n">
         <f aca="false">2*B4</f>
@@ -2073,7 +2096,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B6" s="2" t="n">
         <f aca="false">2*Inputs!B8</f>
@@ -2082,7 +2105,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B7" s="2" t="n">
         <f aca="false">B5+B6</f>
@@ -2091,7 +2114,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B8" s="2" t="str">
         <f aca="false">IF(Inputs!B6&lt;=Inputs!B7,"standard roster: nine rounds, seven on Friday and two on Saturday morning",IF(Inputs!B6&lt;=B5+2,"stretch: stream B runs more Friday rounds, up to "&amp;B5&amp;" rounds across both streams in block one, and Saturday keeps its two",IF(Inputs!B6&lt;=B7,"stretch: stream B runs all Friday rounds and both streams run up to "&amp;Inputs!B8&amp;" Saturday rounds, which moves Saturday presentations back by up to "&amp;(Inputs!B8-1)*Inputs!B3&amp;" minutes","over the two expert days: the Programme Head adds a third chair")))</f>
@@ -2100,7 +2123,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B9" s="2" t="n">
         <f aca="false">COUNTIF(Roster!N4:N12,"swap*")</f>
@@ -2109,7 +2132,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B10" s="2" t="str">
         <f aca="false">IF(B9=0,"no group meets its own sub-problem",B9&amp;" clash: swap within the level or use card 08")</f>
@@ -2118,7 +2141,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B11" s="2" t="n">
         <f aca="false">COUNTIF(Roster!O4:O12,"over*")</f>
@@ -2127,7 +2150,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B12" s="2" t="str">
         <f aca="false">IF(B11=0,"every round ends inside its block",B11&amp;" round runs past the block end")</f>
@@ -2136,11 +2159,47 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B13" s="2" t="str">
         <f aca="false">IF(SUMPRODUCT((COUNTIF(Inputs!C13:C21,Inputs!C13:C21)&gt;1)*1)=0,"every group sits exactly one GD","two groups share a slot: redraw")</f>
         <v>every group sits exactly one GD</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <f aca="false">COUNTIF(Roster!K4:K12,"no group drawn")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <f aca="false">IF(B14=0,"every slot has a group drawn","slots with no group drawn: "&amp;B14&amp;"; check the draw positions on Inputs")</f>
+        <v>every slot has a group drawn</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <f aca="false">COUNTIF(Inputs!C13:C21,"&gt;9")+COUNTIF(Inputs!C13:C21,"&lt;1")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" s="2" t="str">
+        <f aca="false">IF(B16=0,"every draw position is between 1 and 9","draw positions outside 1 to 9: "&amp;B16&amp;"; retype them on Inputs")</f>
+        <v>every draw position is between 1 and 9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W03 D5 workbooks after round 2: the roster's Read me says the trainer types the draw and gives the three swap steps, its clash verdict names all three, its manifest asserts card 10's flag and flips a billing group onto card 10 (11 verdicts, 5 flips), and both manifests open on the question they prove
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014hvr14zDU6tq3n9FYhf2vM
</commit_message>
<xml_diff>
--- a/content/W03/D5/gd/C2_W03_D05_gd_roster_TRAINER.xlsx
+++ b/content/W03/D5/gd/C2_W03_D05_gd_roster_TRAINER.xlsx
@@ -42,7 +42,7 @@
     <t xml:space="preserve">On Monday, replace the sub-problem values on Inputs with the Programme Head's allocation. The values shipped are an example, placed so that the shipped draw shows no clash.</t>
   </si>
   <si>
-    <t xml:space="preserve">At the Friday opening, the Programme Head draws the GD order by lot and types each group's position on Inputs. Slot 1 is the first round; the card each slot carries is fixed on Roster, so complexity climbs with the slot.</t>
+    <t xml:space="preserve">At the Friday opening, the Programme Head draws the GD order by lot, and the trainer types each group's position on Inputs and reads Check before round 1. Slot 1 is the first round; the card each slot carries is fixed on Roster, so complexity climbs with the slot.</t>
   </si>
   <si>
     <t xml:space="preserve">Cards 01 to 04 read for four minutes and discuss for seventeen, cards 05 to 08 read for five and discuss for sixteen, and cards 09 and 10 read for six and discuss for fifteen. Every round is 30 minutes.</t>
@@ -54,7 +54,7 @@
     <t xml:space="preserve">The roster seats nine groups. With more, change the group count on Inputs to read the stretch on Check, and seat each extra round by hand in the time Check names.</t>
   </si>
   <si>
-    <t xml:space="preserve">A clash means swapping the card with the other card of the same level on Roster, if that card's own flag allows, or with the spare, card 08, which is kept from nobody.</t>
+    <t xml:space="preserve">Clear every clash before round 1 with three fixes, tried in order. First, swap the card on Roster with the other card of its level, if neither group would then sit a card it is kept from. Second, give the group card 08, the spare, on Roster, if no other group has it yet. Third, swap the group's draw position on Inputs with the nearest group for which both moves are allowed. The third fix always exists: under either of Monday's allocations, every order in which nine groups can be drawn ends with no clash.</t>
   </si>
   <si>
     <t xml:space="preserve">Inputs</t>
@@ -813,7 +813,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>111</v>
       </c>
       <c r="B10" s="2" t="str">
-        <f aca="false">IF(B9=0,"no group meets its own sub-problem",B9&amp;" clash: swap within the level or use card 08")</f>
+        <f aca="false">IF(B9=0,"no group meets its own sub-problem",B9&amp;" clash: swap within the level, use card 08, or swap two draw positions")</f>
         <v>no group meets its own sub-problem</v>
       </c>
     </row>

</xml_diff>